<commit_message>
Rebuild Canyon Ridge supply chart with HelloData 5-mi unit details
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gzof5jycbxc5BFsHyg4DJw
</commit_message>
<xml_diff>
--- a/CanyonRidge/supply/Canyon_Ridge__Supply_Chart.xlsx
+++ b/CanyonRidge/supply/Canyon_Ridge__Supply_Chart.xlsx
@@ -895,7 +895,7 @@
         <v>0.974453</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>2213</v>
+        <v>2147.615759341101</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
     <row r="24">
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>* 5-Mile radius. Rent ($) = market asking. Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
+          <t>* 5-Mile radius. Rent ($) = HelloData mix-weighted asking where covered, else market asking (CoStar). Proximity (mi) = straight-line distance from the subject. Est. Delivery drives the Supply &amp; Absorption tab's per-window supply (edit it there or here — they are linked). See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
       </c>
     </row>
@@ -2185,10 +2185,10 @@
         <v>1953</v>
       </c>
       <c r="H23" s="48" t="n">
-        <v>1977</v>
+        <v>1944</v>
       </c>
       <c r="I23" s="48">
-        <f>IFERROR('Cash Flow (Annual)'!$F$4,2136)</f>
+        <f>IFERROR('Cash Flow (Annual)'!$F$4,2029)</f>
         <v/>
       </c>
       <c r="J23" s="49">
@@ -2294,10 +2294,10 @@
         <v>1953</v>
       </c>
       <c r="H25" s="48" t="n">
-        <v>1823</v>
+        <v>1795</v>
       </c>
       <c r="I25" s="48">
-        <f>IFERROR('Cash Flow (Annual)'!$F$5,2018)</f>
+        <f>IFERROR('Cash Flow (Annual)'!$F$5,1924)</f>
         <v/>
       </c>
       <c r="J25" s="49">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E66" s="71" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>HD</t>
         </is>
       </c>
     </row>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="E67" s="71" t="inlineStr">
         <is>
-          <t>HD occ + CoStar rents</t>
+          <t>HD</t>
         </is>
       </c>
     </row>
@@ -3806,8 +3806,12 @@
       <c r="L5" s="74" t="n">
         <v>2303</v>
       </c>
-      <c r="M5" s="74" t="n"/>
-      <c r="N5" s="74" t="n"/>
+      <c r="M5" s="74" t="n">
+        <v>2147.615759341101</v>
+      </c>
+      <c r="N5" s="74" t="n">
+        <v>2147.615759341101</v>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>

</xml_diff>